<commit_message>
add 2 files of test
</commit_message>
<xml_diff>
--- a/RL/results_scalar_film_b.xlsx
+++ b/RL/results_scalar_film_b.xlsx
@@ -593,7 +593,7 @@
         <v>75</v>
       </c>
       <c r="U2" t="n">
-        <v>17561.6</v>
+        <v>12333.2</v>
       </c>
       <c r="V2" t="n">
         <v>93.29000000000001</v>
@@ -663,7 +663,7 @@
         <v>3</v>
       </c>
       <c r="U3" t="n">
-        <v>4532.7</v>
+        <v>754.2</v>
       </c>
       <c r="V3" t="n">
         <v>232.81</v>
@@ -733,7 +733,7 @@
         <v>2</v>
       </c>
       <c r="U4" t="n">
-        <v>287</v>
+        <v>160.2</v>
       </c>
       <c r="V4" t="n">
         <v>200.63</v>
@@ -803,7 +803,7 @@
         <v>2</v>
       </c>
       <c r="U5" t="n">
-        <v>568</v>
+        <v>365.7</v>
       </c>
       <c r="V5" t="n">
         <v>200.63</v>
@@ -873,7 +873,7 @@
         <v>1</v>
       </c>
       <c r="U6" t="n">
-        <v>171.2</v>
+        <v>112.1</v>
       </c>
       <c r="V6" t="n">
         <v>164.85</v>
@@ -943,7 +943,7 @@
         <v>1</v>
       </c>
       <c r="U7" t="n">
-        <v>188.6</v>
+        <v>150.3</v>
       </c>
       <c r="V7" t="n">
         <v>163.65</v>
@@ -1013,7 +1013,7 @@
         <v>1</v>
       </c>
       <c r="U8" t="n">
-        <v>739.6</v>
+        <v>425</v>
       </c>
       <c r="V8" t="n">
         <v>162.45</v>
@@ -1083,7 +1083,7 @@
         <v>1</v>
       </c>
       <c r="U9" t="n">
-        <v>577.3</v>
+        <v>137.8</v>
       </c>
       <c r="V9" t="n">
         <v>164.85</v>
@@ -1153,7 +1153,7 @@
         <v>2</v>
       </c>
       <c r="U10" t="n">
-        <v>1050.3</v>
+        <v>544.4</v>
       </c>
       <c r="V10" t="n">
         <v>164.85</v>
@@ -1223,7 +1223,7 @@
         <v>1</v>
       </c>
       <c r="U11" t="n">
-        <v>128.4</v>
+        <v>115.8</v>
       </c>
       <c r="V11" t="n">
         <v>199.43</v>
@@ -1293,7 +1293,7 @@
         <v>1</v>
       </c>
       <c r="U12" t="n">
-        <v>178.8</v>
+        <v>156.5</v>
       </c>
       <c r="V12" t="n">
         <v>198.23</v>
@@ -1363,7 +1363,7 @@
         <v>1</v>
       </c>
       <c r="U13" t="n">
-        <v>470.9</v>
+        <v>321.6</v>
       </c>
       <c r="V13" t="n">
         <v>197.03</v>
@@ -1433,7 +1433,7 @@
         <v>1</v>
       </c>
       <c r="U14" t="n">
-        <v>100.4</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="V14" t="n">
         <v>200.63</v>
@@ -1503,7 +1503,7 @@
         <v>1</v>
       </c>
       <c r="U15" t="n">
-        <v>110</v>
+        <v>90.3</v>
       </c>
       <c r="V15" t="n">
         <v>199.43</v>
@@ -1573,7 +1573,7 @@
         <v>1</v>
       </c>
       <c r="U16" t="n">
-        <v>217.8</v>
+        <v>185.9</v>
       </c>
       <c r="V16" t="n">
         <v>198.23</v>
@@ -1643,7 +1643,7 @@
         <v>2</v>
       </c>
       <c r="U17" t="n">
-        <v>342</v>
+        <v>296</v>
       </c>
       <c r="V17" t="n">
         <v>199.43</v>
@@ -1713,7 +1713,7 @@
         <v>3</v>
       </c>
       <c r="U18" t="n">
-        <v>1133.2</v>
+        <v>872.2</v>
       </c>
       <c r="V18" t="n">
         <v>164.85</v>
@@ -1783,7 +1783,7 @@
         <v>3</v>
       </c>
       <c r="U19" t="n">
-        <v>748.1</v>
+        <v>664.6</v>
       </c>
       <c r="V19" t="n">
         <v>200.63</v>
@@ -1853,7 +1853,7 @@
         <v>1</v>
       </c>
       <c r="U20" t="n">
-        <v>153.8</v>
+        <v>143</v>
       </c>
       <c r="V20" t="n">
         <v>129.07</v>
@@ -1923,7 +1923,7 @@
         <v>75</v>
       </c>
       <c r="U21" t="n">
-        <v>20849.3</v>
+        <v>17887.6</v>
       </c>
       <c r="V21" t="n">
         <v>21.73</v>
@@ -1993,7 +1993,7 @@
         <v>75</v>
       </c>
       <c r="U22" t="n">
-        <v>13444.9</v>
+        <v>13024.8</v>
       </c>
       <c r="V22" t="n">
         <v>57.51</v>
@@ -2063,7 +2063,7 @@
         <v>1</v>
       </c>
       <c r="U23" t="n">
-        <v>186.6</v>
+        <v>231.1</v>
       </c>
       <c r="V23" t="n">
         <v>98.08</v>
@@ -2133,7 +2133,7 @@
         <v>4</v>
       </c>
       <c r="U24" t="n">
-        <v>473.5</v>
+        <v>545.2</v>
       </c>
       <c r="V24" t="n">
         <v>232.81</v>
@@ -2203,7 +2203,7 @@
         <v>4</v>
       </c>
       <c r="U25" t="n">
-        <v>1175.1</v>
+        <v>1110.5</v>
       </c>
       <c r="V25" t="n">
         <v>232.81</v>
@@ -2273,7 +2273,7 @@
         <v>1</v>
       </c>
       <c r="U26" t="n">
-        <v>206.7</v>
+        <v>191.3</v>
       </c>
       <c r="V26" t="n">
         <v>200.63</v>
@@ -2343,7 +2343,7 @@
         <v>2</v>
       </c>
       <c r="U27" t="n">
-        <v>503.1</v>
+        <v>508.5</v>
       </c>
       <c r="V27" t="n">
         <v>200.63</v>
@@ -2413,7 +2413,7 @@
         <v>1</v>
       </c>
       <c r="U28" t="n">
-        <v>138.9</v>
+        <v>139.6</v>
       </c>
       <c r="V28" t="n">
         <v>164.85</v>
@@ -2483,7 +2483,7 @@
         <v>1</v>
       </c>
       <c r="U29" t="n">
-        <v>247</v>
+        <v>245.1</v>
       </c>
       <c r="V29" t="n">
         <v>163.65</v>
@@ -2553,7 +2553,7 @@
         <v>1</v>
       </c>
       <c r="U30" t="n">
-        <v>576</v>
+        <v>577.7</v>
       </c>
       <c r="V30" t="n">
         <v>161.25</v>
@@ -2623,7 +2623,7 @@
         <v>2</v>
       </c>
       <c r="U31" t="n">
-        <v>348.9</v>
+        <v>385.9</v>
       </c>
       <c r="V31" t="n">
         <v>164.85</v>
@@ -2693,7 +2693,7 @@
         <v>3</v>
       </c>
       <c r="U32" t="n">
-        <v>1179.4</v>
+        <v>1077.5</v>
       </c>
       <c r="V32" t="n">
         <v>164.85</v>
@@ -2763,7 +2763,7 @@
         <v>1</v>
       </c>
       <c r="U33" t="n">
-        <v>128.4</v>
+        <v>206.8</v>
       </c>
       <c r="V33" t="n">
         <v>199.43</v>
@@ -2833,7 +2833,7 @@
         <v>1</v>
       </c>
       <c r="U34" t="n">
-        <v>223.3</v>
+        <v>223.8</v>
       </c>
       <c r="V34" t="n">
         <v>198.23</v>
@@ -2903,7 +2903,7 @@
         <v>1</v>
       </c>
       <c r="U35" t="n">
-        <v>421.1</v>
+        <v>403.9</v>
       </c>
       <c r="V35" t="n">
         <v>195.84</v>
@@ -2973,7 +2973,7 @@
         <v>1</v>
       </c>
       <c r="U36" t="n">
-        <v>88.59999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="V36" t="n">
         <v>200.63</v>
@@ -3043,7 +3043,7 @@
         <v>1</v>
       </c>
       <c r="U37" t="n">
-        <v>141</v>
+        <v>135.6</v>
       </c>
       <c r="V37" t="n">
         <v>199.43</v>
@@ -3113,7 +3113,7 @@
         <v>1</v>
       </c>
       <c r="U38" t="n">
-        <v>289</v>
+        <v>274.8</v>
       </c>
       <c r="V38" t="n">
         <v>197.03</v>
@@ -3183,7 +3183,7 @@
         <v>2</v>
       </c>
       <c r="U39" t="n">
-        <v>573.8</v>
+        <v>551.1</v>
       </c>
       <c r="V39" t="n">
         <v>199.43</v>
@@ -3253,7 +3253,7 @@
         <v>3</v>
       </c>
       <c r="U40" t="n">
-        <v>579.9</v>
+        <v>466.6</v>
       </c>
       <c r="V40" t="n">
         <v>200.63</v>
@@ -3323,7 +3323,7 @@
         <v>1</v>
       </c>
       <c r="U41" t="n">
-        <v>133.8</v>
+        <v>124</v>
       </c>
       <c r="V41" t="n">
         <v>164.85</v>
@@ -3393,7 +3393,7 @@
         <v>1</v>
       </c>
       <c r="U42" t="n">
-        <v>246</v>
+        <v>235.6</v>
       </c>
       <c r="V42" t="n">
         <v>129.07</v>
@@ -3463,7 +3463,7 @@
         <v>1</v>
       </c>
       <c r="U43" t="n">
-        <v>123.8</v>
+        <v>113.3</v>
       </c>
       <c r="V43" t="n">
         <v>166.05</v>
@@ -3533,7 +3533,7 @@
         <v>1</v>
       </c>
       <c r="U44" t="n">
-        <v>262.5</v>
+        <v>177.1</v>
       </c>
       <c r="V44" t="n">
         <v>131.47</v>
@@ -3603,7 +3603,7 @@
         <v>1</v>
       </c>
       <c r="U45" t="n">
-        <v>270.7</v>
+        <v>268.5</v>
       </c>
       <c r="V45" t="n">
         <v>153.29</v>
@@ -3673,7 +3673,7 @@
         <v>4</v>
       </c>
       <c r="U46" t="n">
-        <v>984.2</v>
+        <v>938.2</v>
       </c>
       <c r="V46" t="n">
         <v>292.81</v>
@@ -3743,7 +3743,7 @@
         <v>2</v>
       </c>
       <c r="U47" t="n">
-        <v>178.3</v>
+        <v>177</v>
       </c>
       <c r="V47" t="n">
         <v>260.63</v>
@@ -3813,7 +3813,7 @@
         <v>3</v>
       </c>
       <c r="U48" t="n">
-        <v>502.8</v>
+        <v>488</v>
       </c>
       <c r="V48" t="n">
         <v>260.63</v>
@@ -3883,7 +3883,7 @@
         <v>1</v>
       </c>
       <c r="U49" t="n">
-        <v>127.7</v>
+        <v>122.8</v>
       </c>
       <c r="V49" t="n">
         <v>224.85</v>
@@ -3953,7 +3953,7 @@
         <v>1</v>
       </c>
       <c r="U50" t="n">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="V50" t="n">
         <v>223.65</v>
@@ -4023,7 +4023,7 @@
         <v>1</v>
       </c>
       <c r="U51" t="n">
-        <v>493.5</v>
+        <v>461.4</v>
       </c>
       <c r="V51" t="n">
         <v>222.45</v>
@@ -4093,7 +4093,7 @@
         <v>1</v>
       </c>
       <c r="U52" t="n">
-        <v>169.5</v>
+        <v>150.8</v>
       </c>
       <c r="V52" t="n">
         <v>224.85</v>
@@ -4163,7 +4163,7 @@
         <v>2</v>
       </c>
       <c r="U53" t="n">
-        <v>662.2</v>
+        <v>612.3</v>
       </c>
       <c r="V53" t="n">
         <v>224.85</v>
@@ -4233,7 +4233,7 @@
         <v>1</v>
       </c>
       <c r="U54" t="n">
-        <v>113</v>
+        <v>114.5</v>
       </c>
       <c r="V54" t="n">
         <v>259.43</v>
@@ -4303,7 +4303,7 @@
         <v>1</v>
       </c>
       <c r="U55" t="n">
-        <v>145.1</v>
+        <v>146.5</v>
       </c>
       <c r="V55" t="n">
         <v>258.23</v>
@@ -4373,7 +4373,7 @@
         <v>1</v>
       </c>
       <c r="U56" t="n">
-        <v>368</v>
+        <v>353.2</v>
       </c>
       <c r="V56" t="n">
         <v>257.03</v>
@@ -4443,7 +4443,7 @@
         <v>1</v>
       </c>
       <c r="U57" t="n">
-        <v>101.1</v>
+        <v>86.7</v>
       </c>
       <c r="V57" t="n">
         <v>260.63</v>
@@ -4513,7 +4513,7 @@
         <v>1</v>
       </c>
       <c r="U58" t="n">
-        <v>111.1</v>
+        <v>103.4</v>
       </c>
       <c r="V58" t="n">
         <v>259.43</v>
@@ -4583,7 +4583,7 @@
         <v>1</v>
       </c>
       <c r="U59" t="n">
-        <v>223.9</v>
+        <v>222.5</v>
       </c>
       <c r="V59" t="n">
         <v>258.23</v>
@@ -4653,7 +4653,7 @@
         <v>3</v>
       </c>
       <c r="U60" t="n">
-        <v>439.2</v>
+        <v>446.3</v>
       </c>
       <c r="V60" t="n">
         <v>224.85</v>
@@ -4723,7 +4723,7 @@
         <v>2</v>
       </c>
       <c r="U61" t="n">
-        <v>738</v>
+        <v>707.2</v>
       </c>
       <c r="V61" t="n">
         <v>259.43</v>
@@ -4793,7 +4793,7 @@
         <v>4</v>
       </c>
       <c r="U62" t="n">
-        <v>926.5</v>
+        <v>910.6</v>
       </c>
       <c r="V62" t="n">
         <v>260.63</v>
@@ -4863,7 +4863,7 @@
         <v>1</v>
       </c>
       <c r="U63" t="n">
-        <v>156.6</v>
+        <v>164.1</v>
       </c>
       <c r="V63" t="n">
         <v>189.07</v>
@@ -4933,7 +4933,7 @@
         <v>75</v>
       </c>
       <c r="U64" t="n">
-        <v>52031.9</v>
+        <v>57641.7</v>
       </c>
       <c r="V64" t="n">
         <v>80.53</v>
@@ -5003,7 +5003,7 @@
         <v>5</v>
       </c>
       <c r="U65" t="n">
-        <v>2432.8</v>
+        <v>2125.6</v>
       </c>
       <c r="V65" t="n">
         <v>113.92</v>
@@ -5073,7 +5073,7 @@
         <v>1</v>
       </c>
       <c r="U66" t="n">
-        <v>255.6</v>
+        <v>250.4</v>
       </c>
       <c r="V66" t="n">
         <v>158.08</v>
@@ -5143,7 +5143,7 @@
         <v>3</v>
       </c>
       <c r="U67" t="n">
-        <v>464.9</v>
+        <v>523.4</v>
       </c>
       <c r="V67" t="n">
         <v>292.81</v>
@@ -5213,7 +5213,7 @@
         <v>4</v>
       </c>
       <c r="U68" t="n">
-        <v>1197.7</v>
+        <v>1228.4</v>
       </c>
       <c r="V68" t="n">
         <v>292.81</v>
@@ -5283,7 +5283,7 @@
         <v>1</v>
       </c>
       <c r="U69" t="n">
-        <v>194.2</v>
+        <v>217.5</v>
       </c>
       <c r="V69" t="n">
         <v>260.63</v>
@@ -5353,7 +5353,7 @@
         <v>2</v>
       </c>
       <c r="U70" t="n">
-        <v>514</v>
+        <v>561.8</v>
       </c>
       <c r="V70" t="n">
         <v>260.63</v>
@@ -5423,7 +5423,7 @@
         <v>1</v>
       </c>
       <c r="U71" t="n">
-        <v>257.7</v>
+        <v>274.9</v>
       </c>
       <c r="V71" t="n">
         <v>224.85</v>
@@ -5493,7 +5493,7 @@
         <v>1</v>
       </c>
       <c r="U72" t="n">
-        <v>232.7</v>
+        <v>273.7</v>
       </c>
       <c r="V72" t="n">
         <v>223.65</v>
@@ -5563,7 +5563,7 @@
         <v>1</v>
       </c>
       <c r="U73" t="n">
-        <v>532.7</v>
+        <v>574.5</v>
       </c>
       <c r="V73" t="n">
         <v>221.25</v>
@@ -5633,7 +5633,7 @@
         <v>3</v>
       </c>
       <c r="U74" t="n">
-        <v>411.9</v>
+        <v>499.6</v>
       </c>
       <c r="V74" t="n">
         <v>224.85</v>
@@ -5703,7 +5703,7 @@
         <v>2</v>
       </c>
       <c r="U75" t="n">
-        <v>872.7</v>
+        <v>927.8</v>
       </c>
       <c r="V75" t="n">
         <v>224.85</v>
@@ -5773,7 +5773,7 @@
         <v>1</v>
       </c>
       <c r="U76" t="n">
-        <v>123.7</v>
+        <v>146</v>
       </c>
       <c r="V76" t="n">
         <v>259.43</v>
@@ -5843,7 +5843,7 @@
         <v>1</v>
       </c>
       <c r="U77" t="n">
-        <v>204.8</v>
+        <v>255.7</v>
       </c>
       <c r="V77" t="n">
         <v>258.23</v>
@@ -5913,7 +5913,7 @@
         <v>1</v>
       </c>
       <c r="U78" t="n">
-        <v>412.7</v>
+        <v>455</v>
       </c>
       <c r="V78" t="n">
         <v>255.84</v>
@@ -5983,7 +5983,7 @@
         <v>1</v>
       </c>
       <c r="U79" t="n">
-        <v>89.09999999999999</v>
+        <v>110.5</v>
       </c>
       <c r="V79" t="n">
         <v>260.63</v>
@@ -6053,7 +6053,7 @@
         <v>1</v>
       </c>
       <c r="U80" t="n">
-        <v>129.2</v>
+        <v>171.7</v>
       </c>
       <c r="V80" t="n">
         <v>259.43</v>
@@ -6123,7 +6123,7 @@
         <v>1</v>
       </c>
       <c r="U81" t="n">
-        <v>260.3</v>
+        <v>335</v>
       </c>
       <c r="V81" t="n">
         <v>257.03</v>
@@ -6193,7 +6193,7 @@
         <v>2</v>
       </c>
       <c r="U82" t="n">
-        <v>550</v>
+        <v>641.2</v>
       </c>
       <c r="V82" t="n">
         <v>259.43</v>
@@ -6263,7 +6263,7 @@
         <v>3</v>
       </c>
       <c r="U83" t="n">
-        <v>475.8</v>
+        <v>566.9</v>
       </c>
       <c r="V83" t="n">
         <v>260.63</v>
@@ -6333,7 +6333,7 @@
         <v>1</v>
       </c>
       <c r="U84" t="n">
-        <v>121.2</v>
+        <v>149.2</v>
       </c>
       <c r="V84" t="n">
         <v>224.85</v>
@@ -6403,7 +6403,7 @@
         <v>1</v>
       </c>
       <c r="U85" t="n">
-        <v>246</v>
+        <v>274.8</v>
       </c>
       <c r="V85" t="n">
         <v>189.07</v>
@@ -6473,7 +6473,7 @@
         <v>1</v>
       </c>
       <c r="U86" t="n">
-        <v>104.9</v>
+        <v>144.7</v>
       </c>
       <c r="V86" t="n">
         <v>226.05</v>
@@ -6543,7 +6543,7 @@
         <v>1</v>
       </c>
       <c r="U87" t="n">
-        <v>163.1</v>
+        <v>206.7</v>
       </c>
       <c r="V87" t="n">
         <v>191.47</v>
@@ -6613,7 +6613,7 @@
         <v>1</v>
       </c>
       <c r="U88" t="n">
-        <v>256.3</v>
+        <v>299.2</v>
       </c>
       <c r="V88" t="n">
         <v>999853.29</v>
@@ -6683,7 +6683,7 @@
         <v>3</v>
       </c>
       <c r="U89" t="n">
-        <v>720.6</v>
+        <v>895</v>
       </c>
       <c r="V89" t="n">
         <v>999992.8100000001</v>
@@ -6753,7 +6753,7 @@
         <v>1</v>
       </c>
       <c r="U90" t="n">
-        <v>118.5</v>
+        <v>162.4</v>
       </c>
       <c r="V90" t="n">
         <v>999960.63</v>
@@ -6823,7 +6823,7 @@
         <v>3</v>
       </c>
       <c r="U91" t="n">
-        <v>454.5</v>
+        <v>571.2</v>
       </c>
       <c r="V91" t="n">
         <v>999960.63</v>
@@ -6893,7 +6893,7 @@
         <v>1</v>
       </c>
       <c r="U92" t="n">
-        <v>120.8</v>
+        <v>128.9</v>
       </c>
       <c r="V92" t="n">
         <v>999924.85</v>
@@ -6963,7 +6963,7 @@
         <v>1</v>
       </c>
       <c r="U93" t="n">
-        <v>160.3</v>
+        <v>191</v>
       </c>
       <c r="V93" t="n">
         <v>999923.65</v>
@@ -7033,7 +7033,7 @@
         <v>1</v>
       </c>
       <c r="U94" t="n">
-        <v>489</v>
+        <v>498.2</v>
       </c>
       <c r="V94" t="n">
         <v>999922.45</v>
@@ -7103,7 +7103,7 @@
         <v>1</v>
       </c>
       <c r="U95" t="n">
-        <v>157.1</v>
+        <v>194.7</v>
       </c>
       <c r="V95" t="n">
         <v>999924.85</v>
@@ -7173,7 +7173,7 @@
         <v>2</v>
       </c>
       <c r="U96" t="n">
-        <v>627.6</v>
+        <v>692.2</v>
       </c>
       <c r="V96" t="n">
         <v>999924.85</v>
@@ -7243,7 +7243,7 @@
         <v>1</v>
       </c>
       <c r="U97" t="n">
-        <v>103.9</v>
+        <v>107.1</v>
       </c>
       <c r="V97" t="n">
         <v>999959.4300000001</v>
@@ -7313,7 +7313,7 @@
         <v>1</v>
       </c>
       <c r="U98" t="n">
-        <v>142.7</v>
+        <v>142.1</v>
       </c>
       <c r="V98" t="n">
         <v>999958.23</v>
@@ -7383,7 +7383,7 @@
         <v>1</v>
       </c>
       <c r="U99" t="n">
-        <v>363.6</v>
+        <v>379.7</v>
       </c>
       <c r="V99" t="n">
         <v>999957.03</v>
@@ -7453,7 +7453,7 @@
         <v>1</v>
       </c>
       <c r="U100" t="n">
-        <v>90.3</v>
+        <v>87.2</v>
       </c>
       <c r="V100" t="n">
         <v>999960.63</v>
@@ -7523,7 +7523,7 @@
         <v>1</v>
       </c>
       <c r="U101" t="n">
-        <v>104.3</v>
+        <v>102.7</v>
       </c>
       <c r="V101" t="n">
         <v>999959.4300000001</v>
@@ -7593,7 +7593,7 @@
         <v>1</v>
       </c>
       <c r="U102" t="n">
-        <v>209.3</v>
+        <v>209.6</v>
       </c>
       <c r="V102" t="n">
         <v>999958.23</v>
@@ -7663,7 +7663,7 @@
         <v>3</v>
       </c>
       <c r="U103" t="n">
-        <v>412.2</v>
+        <v>400.3</v>
       </c>
       <c r="V103" t="n">
         <v>999924.85</v>
@@ -7733,7 +7733,7 @@
         <v>3</v>
       </c>
       <c r="U104" t="n">
-        <v>981.5</v>
+        <v>908.5</v>
       </c>
       <c r="V104" t="n">
         <v>999924.85</v>
@@ -7803,7 +7803,7 @@
         <v>4</v>
       </c>
       <c r="U105" t="n">
-        <v>890.2</v>
+        <v>921.5</v>
       </c>
       <c r="V105" t="n">
         <v>999960.63</v>
@@ -7873,7 +7873,7 @@
         <v>1</v>
       </c>
       <c r="U106" t="n">
-        <v>168.7</v>
+        <v>167.7</v>
       </c>
       <c r="V106" t="n">
         <v>999889.0699999999</v>
@@ -7943,7 +7943,7 @@
         <v>75</v>
       </c>
       <c r="U107" t="n">
-        <v>26180.7</v>
+        <v>19735.8</v>
       </c>
       <c r="V107" t="n">
         <v>999781.73</v>
@@ -8013,7 +8013,7 @@
         <v>5</v>
       </c>
       <c r="U108" t="n">
-        <v>1941</v>
+        <v>1718.8</v>
       </c>
       <c r="V108" t="n">
         <v>999813.92</v>
@@ -8083,7 +8083,7 @@
         <v>1</v>
       </c>
       <c r="U109" t="n">
-        <v>217.3</v>
+        <v>209.9</v>
       </c>
       <c r="V109" t="n">
         <v>999858.08</v>
@@ -8153,7 +8153,7 @@
         <v>3</v>
       </c>
       <c r="U110" t="n">
-        <v>517.6</v>
+        <v>446</v>
       </c>
       <c r="V110" t="n">
         <v>999992.8100000001</v>
@@ -8223,7 +8223,7 @@
         <v>4</v>
       </c>
       <c r="U111" t="n">
-        <v>1114</v>
+        <v>1071.6</v>
       </c>
       <c r="V111" t="n">
         <v>999992.8100000001</v>
@@ -8293,7 +8293,7 @@
         <v>2</v>
       </c>
       <c r="U112" t="n">
-        <v>263.4</v>
+        <v>256.5</v>
       </c>
       <c r="V112" t="n">
         <v>999960.63</v>
@@ -8363,7 +8363,7 @@
         <v>2</v>
       </c>
       <c r="U113" t="n">
-        <v>525.5</v>
+        <v>486.8</v>
       </c>
       <c r="V113" t="n">
         <v>999960.63</v>
@@ -8433,7 +8433,7 @@
         <v>1</v>
       </c>
       <c r="U114" t="n">
-        <v>144.6</v>
+        <v>137.8</v>
       </c>
       <c r="V114" t="n">
         <v>999924.85</v>
@@ -8503,7 +8503,7 @@
         <v>1</v>
       </c>
       <c r="U115" t="n">
-        <v>266.6</v>
+        <v>247.6</v>
       </c>
       <c r="V115" t="n">
         <v>999923.65</v>
@@ -8573,7 +8573,7 @@
         <v>1</v>
       </c>
       <c r="U116" t="n">
-        <v>718.6</v>
+        <v>488.4</v>
       </c>
       <c r="V116" t="n">
         <v>999921.25</v>
@@ -8643,7 +8643,7 @@
         <v>2</v>
       </c>
       <c r="U117" t="n">
-        <v>357.4</v>
+        <v>340.7</v>
       </c>
       <c r="V117" t="n">
         <v>999924.85</v>
@@ -8713,7 +8713,7 @@
         <v>2</v>
       </c>
       <c r="U118" t="n">
-        <v>1029.4</v>
+        <v>869</v>
       </c>
       <c r="V118" t="n">
         <v>999924.85</v>
@@ -8783,7 +8783,7 @@
         <v>1</v>
       </c>
       <c r="U119" t="n">
-        <v>133.8</v>
+        <v>124.4</v>
       </c>
       <c r="V119" t="n">
         <v>999959.4300000001</v>
@@ -8853,7 +8853,7 @@
         <v>1</v>
       </c>
       <c r="U120" t="n">
-        <v>227.9</v>
+        <v>214.5</v>
       </c>
       <c r="V120" t="n">
         <v>999958.23</v>
@@ -8923,7 +8923,7 @@
         <v>1</v>
       </c>
       <c r="U121" t="n">
-        <v>411.1</v>
+        <v>406.1</v>
       </c>
       <c r="V121" t="n">
         <v>999955.84</v>
@@ -8993,7 +8993,7 @@
         <v>1</v>
       </c>
       <c r="U122" t="n">
-        <v>92.3</v>
+        <v>89.5</v>
       </c>
       <c r="V122" t="n">
         <v>999960.63</v>
@@ -9063,7 +9063,7 @@
         <v>1</v>
       </c>
       <c r="U123" t="n">
-        <v>142.7</v>
+        <v>127.8</v>
       </c>
       <c r="V123" t="n">
         <v>999959.4300000001</v>
@@ -9133,7 +9133,7 @@
         <v>1</v>
       </c>
       <c r="U124" t="n">
-        <v>291</v>
+        <v>263.5</v>
       </c>
       <c r="V124" t="n">
         <v>999957.03</v>
@@ -9203,7 +9203,7 @@
         <v>2</v>
       </c>
       <c r="U125" t="n">
-        <v>590.2</v>
+        <v>546.7</v>
       </c>
       <c r="V125" t="n">
         <v>999959.4300000001</v>
@@ -9273,7 +9273,7 @@
         <v>3</v>
       </c>
       <c r="U126" t="n">
-        <v>581</v>
+        <v>473.1</v>
       </c>
       <c r="V126" t="n">
         <v>999960.63</v>
@@ -9343,7 +9343,7 @@
         <v>1</v>
       </c>
       <c r="U127" t="n">
-        <v>161.9</v>
+        <v>128.9</v>
       </c>
       <c r="V127" t="n">
         <v>999924.85</v>
@@ -9413,7 +9413,7 @@
         <v>1</v>
       </c>
       <c r="U128" t="n">
-        <v>396.6</v>
+        <v>235.8</v>
       </c>
       <c r="V128" t="n">
         <v>999889.0699999999</v>
@@ -9483,7 +9483,7 @@
         <v>1</v>
       </c>
       <c r="U129" t="n">
-        <v>267.2</v>
+        <v>113.9</v>
       </c>
       <c r="V129" t="n">
         <v>999926.05</v>
@@ -9553,7 +9553,7 @@
         <v>1</v>
       </c>
       <c r="U130" t="n">
-        <v>749.1</v>
+        <v>178.6</v>
       </c>
       <c r="V130" t="n">
         <v>999891.47</v>

</xml_diff>